<commit_message>
run week 3 bets
</commit_message>
<xml_diff>
--- a/betting_lines_open_2026.xlsx
+++ b/betting_lines_open_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\OneDrive - Hunter - CUNY\Documents\Football-DNA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7116C22-0578-441F-971C-FBEEBA9A4EB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AE96F25-9EEB-4815-9552-0F36EB6C92EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="1" xr2:uid="{38E66C5D-58C4-4402-8F4D-2FF7B602BD04}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="11370" firstSheet="1" activeTab="1" xr2:uid="{38E66C5D-58C4-4402-8F4D-2FF7B602BD04}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 11" sheetId="9" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="53">
   <si>
     <t>game</t>
   </si>
@@ -148,6 +148,54 @@
   </si>
   <si>
     <t>NYG_LA</t>
+  </si>
+  <si>
+    <t>ATL_GB</t>
+  </si>
+  <si>
+    <t>SEA_WAS</t>
+  </si>
+  <si>
+    <t>CIN_PIT</t>
+  </si>
+  <si>
+    <t>NYJ_DET</t>
+  </si>
+  <si>
+    <t>TEN_NYG</t>
+  </si>
+  <si>
+    <t>NE_JAX</t>
+  </si>
+  <si>
+    <t>KC_MIA</t>
+  </si>
+  <si>
+    <t>HOU_IND</t>
+  </si>
+  <si>
+    <t>CAR_CLE</t>
+  </si>
+  <si>
+    <t>LAC_BUF</t>
+  </si>
+  <si>
+    <t>MIN_TB</t>
+  </si>
+  <si>
+    <t>ARI_SF</t>
+  </si>
+  <si>
+    <t>LV_NO</t>
+  </si>
+  <si>
+    <t>BAL_DAL</t>
+  </si>
+  <si>
+    <t>LA_DEN</t>
+  </si>
+  <si>
+    <t>PHI_CHI</t>
   </si>
 </sst>
 </file>
@@ -705,7 +753,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FD36202-D83D-42C3-9E22-D680F63FC59E}">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -946,6 +994,230 @@
         <v>8.5</v>
       </c>
     </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18">
+        <v>3</v>
+      </c>
+      <c r="B18" t="s">
+        <v>37</v>
+      </c>
+      <c r="C18">
+        <v>46.5</v>
+      </c>
+      <c r="D18">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>3</v>
+      </c>
+      <c r="B19" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19">
+        <v>46.5</v>
+      </c>
+      <c r="D19">
+        <v>-3.5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20">
+        <v>3</v>
+      </c>
+      <c r="B20" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20">
+        <v>47.5</v>
+      </c>
+      <c r="D20">
+        <v>-1.5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>3</v>
+      </c>
+      <c r="B21" t="s">
+        <v>40</v>
+      </c>
+      <c r="C21">
+        <v>45.5</v>
+      </c>
+      <c r="D21">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <v>3</v>
+      </c>
+      <c r="B22" t="s">
+        <v>41</v>
+      </c>
+      <c r="C22">
+        <v>45.5</v>
+      </c>
+      <c r="D22">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <v>3</v>
+      </c>
+      <c r="B23" t="s">
+        <v>42</v>
+      </c>
+      <c r="C23">
+        <v>45.5</v>
+      </c>
+      <c r="D23">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24">
+        <v>3</v>
+      </c>
+      <c r="B24" t="s">
+        <v>43</v>
+      </c>
+      <c r="C24">
+        <v>44.5</v>
+      </c>
+      <c r="D24">
+        <v>-7</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25">
+        <v>3</v>
+      </c>
+      <c r="B25" t="s">
+        <v>44</v>
+      </c>
+      <c r="C25">
+        <v>45.5</v>
+      </c>
+      <c r="D25">
+        <v>-1.5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26">
+        <v>3</v>
+      </c>
+      <c r="B26" t="s">
+        <v>45</v>
+      </c>
+      <c r="C26">
+        <v>39.5</v>
+      </c>
+      <c r="D26">
+        <v>-1.5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27">
+        <v>3</v>
+      </c>
+      <c r="B27" t="s">
+        <v>46</v>
+      </c>
+      <c r="C27">
+        <v>48.5</v>
+      </c>
+      <c r="D27">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28">
+        <v>3</v>
+      </c>
+      <c r="B28" t="s">
+        <v>47</v>
+      </c>
+      <c r="C28">
+        <v>44.5</v>
+      </c>
+      <c r="D28">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>3</v>
+      </c>
+      <c r="B29" t="s">
+        <v>48</v>
+      </c>
+      <c r="C29">
+        <v>46.5</v>
+      </c>
+      <c r="D29">
+        <v>11.5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30">
+        <v>3</v>
+      </c>
+      <c r="B30" t="s">
+        <v>49</v>
+      </c>
+      <c r="C30">
+        <v>42.5</v>
+      </c>
+      <c r="D30">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <v>3</v>
+      </c>
+      <c r="B31" t="s">
+        <v>50</v>
+      </c>
+      <c r="C31">
+        <v>50.5</v>
+      </c>
+      <c r="D31">
+        <v>-2.5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <v>3</v>
+      </c>
+      <c r="B32" t="s">
+        <v>51</v>
+      </c>
+      <c r="C32">
+        <v>45.5</v>
+      </c>
+      <c r="D32">
+        <v>-2.5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33">
+        <v>3</v>
+      </c>
+      <c r="B33" t="s">
+        <v>52</v>
+      </c>
+      <c r="C33">
+        <v>46.5</v>
+      </c>
+      <c r="D33">
+        <v>1.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
initial week 5 run
</commit_message>
<xml_diff>
--- a/betting_lines_open_2026.xlsx
+++ b/betting_lines_open_2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\OneDrive - Hunter - CUNY\Documents\Football-DNA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3990ED3B-32D8-44FE-9BBD-59DD11E831F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{290EF09A-FA49-450A-AA1D-4C95A86AFC18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="11370" firstSheet="1" activeTab="1" xr2:uid="{38E66C5D-58C4-4402-8F4D-2FF7B602BD04}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="84">
   <si>
     <t>game</t>
   </si>
@@ -244,6 +244,51 @@
   </si>
   <si>
     <t>ATL_NO</t>
+  </si>
+  <si>
+    <t>TB_DAL</t>
+  </si>
+  <si>
+    <t>PHI_JAX</t>
+  </si>
+  <si>
+    <t>IND_PIT</t>
+  </si>
+  <si>
+    <t>MIN_NO</t>
+  </si>
+  <si>
+    <t>CLE_NYJ</t>
+  </si>
+  <si>
+    <t>CIN_MIA</t>
+  </si>
+  <si>
+    <t>LV_NE</t>
+  </si>
+  <si>
+    <t>NYG_WAS</t>
+  </si>
+  <si>
+    <t>HOU_TEN</t>
+  </si>
+  <si>
+    <t>CHI_GB</t>
+  </si>
+  <si>
+    <t>DEN_LAC</t>
+  </si>
+  <si>
+    <t>SF_SEA</t>
+  </si>
+  <si>
+    <t>DET_ARI</t>
+  </si>
+  <si>
+    <t>BAL_ATL</t>
+  </si>
+  <si>
+    <t>BUF_LA</t>
   </si>
 </sst>
 </file>
@@ -801,7 +846,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FD36202-D83D-42C3-9E22-D680F63FC59E}">
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -1490,6 +1535,216 @@
         <v>2.5</v>
       </c>
     </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A50">
+        <v>5</v>
+      </c>
+      <c r="B50" t="s">
+        <v>69</v>
+      </c>
+      <c r="C50">
+        <v>52.5</v>
+      </c>
+      <c r="D50">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A51">
+        <v>5</v>
+      </c>
+      <c r="B51" t="s">
+        <v>70</v>
+      </c>
+      <c r="C51">
+        <v>43.5</v>
+      </c>
+      <c r="D51">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A52">
+        <v>5</v>
+      </c>
+      <c r="B52" t="s">
+        <v>71</v>
+      </c>
+      <c r="C52">
+        <v>47.5</v>
+      </c>
+      <c r="D52">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A53">
+        <v>5</v>
+      </c>
+      <c r="B53" t="s">
+        <v>72</v>
+      </c>
+      <c r="C53">
+        <v>44.5</v>
+      </c>
+      <c r="D53">
+        <v>-1.5</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A54">
+        <v>5</v>
+      </c>
+      <c r="B54" t="s">
+        <v>73</v>
+      </c>
+      <c r="C54">
+        <v>39.5</v>
+      </c>
+      <c r="D54">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A55">
+        <v>5</v>
+      </c>
+      <c r="B55" t="s">
+        <v>74</v>
+      </c>
+      <c r="C55">
+        <v>49.5</v>
+      </c>
+      <c r="D55">
+        <v>-8.5</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A56">
+        <v>5</v>
+      </c>
+      <c r="B56" t="s">
+        <v>75</v>
+      </c>
+      <c r="C56">
+        <v>44.5</v>
+      </c>
+      <c r="D56">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A57">
+        <v>5</v>
+      </c>
+      <c r="B57" t="s">
+        <v>76</v>
+      </c>
+      <c r="C57">
+        <v>48.5</v>
+      </c>
+      <c r="D57">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A58">
+        <v>5</v>
+      </c>
+      <c r="B58" t="s">
+        <v>77</v>
+      </c>
+      <c r="C58">
+        <v>43.5</v>
+      </c>
+      <c r="D58">
+        <v>-3.5</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A59">
+        <v>5</v>
+      </c>
+      <c r="B59" t="s">
+        <v>78</v>
+      </c>
+      <c r="C59">
+        <v>49.5</v>
+      </c>
+      <c r="D59">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A60">
+        <v>5</v>
+      </c>
+      <c r="B60" t="s">
+        <v>79</v>
+      </c>
+      <c r="C60">
+        <v>44.5</v>
+      </c>
+      <c r="D60">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A61">
+        <v>5</v>
+      </c>
+      <c r="B61" t="s">
+        <v>80</v>
+      </c>
+      <c r="C61">
+        <v>48.5</v>
+      </c>
+      <c r="D61">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A62">
+        <v>5</v>
+      </c>
+      <c r="B62" t="s">
+        <v>81</v>
+      </c>
+      <c r="C62">
+        <v>49.5</v>
+      </c>
+      <c r="D62">
+        <v>-8.5</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A63">
+        <v>5</v>
+      </c>
+      <c r="B63" t="s">
+        <v>82</v>
+      </c>
+      <c r="C63">
+        <v>48.5</v>
+      </c>
+      <c r="D63">
+        <v>-4.5</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A64">
+        <v>5</v>
+      </c>
+      <c r="B64" t="s">
+        <v>83</v>
+      </c>
+      <c r="C64">
+        <v>53.5</v>
+      </c>
+      <c r="D64">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
initial week 6 run
</commit_message>
<xml_diff>
--- a/betting_lines_open_2026.xlsx
+++ b/betting_lines_open_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\OneDrive - Hunter - CUNY\Documents\Football-DNA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{290EF09A-FA49-450A-AA1D-4C95A86AFC18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0264E3A-CC1D-4478-8803-563321D1F0B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="11370" firstSheet="1" activeTab="1" xr2:uid="{38E66C5D-58C4-4402-8F4D-2FF7B602BD04}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" firstSheet="1" activeTab="1" xr2:uid="{38E66C5D-58C4-4402-8F4D-2FF7B602BD04}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 11" sheetId="9" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="98">
   <si>
     <t>game</t>
   </si>
@@ -289,6 +289,48 @@
   </si>
   <si>
     <t>BUF_LA</t>
+  </si>
+  <si>
+    <t>SEA_DEN</t>
+  </si>
+  <si>
+    <t>HOU_JAX</t>
+  </si>
+  <si>
+    <t>NYJ_NE</t>
+  </si>
+  <si>
+    <t>PIT_TB</t>
+  </si>
+  <si>
+    <t>BAL_CLE</t>
+  </si>
+  <si>
+    <t>CHI_ATL</t>
+  </si>
+  <si>
+    <t>TEN_IND</t>
+  </si>
+  <si>
+    <t>CAR_PHI</t>
+  </si>
+  <si>
+    <t>NO_NYG</t>
+  </si>
+  <si>
+    <t>ARI_LA</t>
+  </si>
+  <si>
+    <t>BUF_LV</t>
+  </si>
+  <si>
+    <t>LAC_KC</t>
+  </si>
+  <si>
+    <t>DAL_GB</t>
+  </si>
+  <si>
+    <t>WAS_SF</t>
   </si>
 </sst>
 </file>
@@ -846,7 +888,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FD36202-D83D-42C3-9E22-D680F63FC59E}">
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:D78"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -1745,6 +1787,202 @@
         <v>3</v>
       </c>
     </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A65">
+        <v>6</v>
+      </c>
+      <c r="B65" t="s">
+        <v>84</v>
+      </c>
+      <c r="C65">
+        <v>43.5</v>
+      </c>
+      <c r="D65">
+        <v>-2.5</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A66">
+        <v>6</v>
+      </c>
+      <c r="B66" t="s">
+        <v>85</v>
+      </c>
+      <c r="C66">
+        <v>41.5</v>
+      </c>
+      <c r="D66">
+        <v>-1.5</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A67">
+        <v>6</v>
+      </c>
+      <c r="B67" t="s">
+        <v>86</v>
+      </c>
+      <c r="C67">
+        <v>42.5</v>
+      </c>
+      <c r="D67">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A68">
+        <v>6</v>
+      </c>
+      <c r="B68" t="s">
+        <v>87</v>
+      </c>
+      <c r="C68">
+        <v>45.5</v>
+      </c>
+      <c r="D68">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A69">
+        <v>6</v>
+      </c>
+      <c r="B69" t="s">
+        <v>88</v>
+      </c>
+      <c r="C69">
+        <v>44.5</v>
+      </c>
+      <c r="D69">
+        <v>-6.5</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A70">
+        <v>6</v>
+      </c>
+      <c r="B70" t="s">
+        <v>89</v>
+      </c>
+      <c r="C70">
+        <v>47.5</v>
+      </c>
+      <c r="D70">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A71">
+        <v>6</v>
+      </c>
+      <c r="B71" t="s">
+        <v>90</v>
+      </c>
+      <c r="C71">
+        <v>48.5</v>
+      </c>
+      <c r="D71">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A72">
+        <v>6</v>
+      </c>
+      <c r="B72" t="s">
+        <v>91</v>
+      </c>
+      <c r="C72">
+        <v>43.5</v>
+      </c>
+      <c r="D72">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A73">
+        <v>6</v>
+      </c>
+      <c r="B73" t="s">
+        <v>92</v>
+      </c>
+      <c r="C73">
+        <v>45.5</v>
+      </c>
+      <c r="D73">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A74">
+        <v>6</v>
+      </c>
+      <c r="B74" t="s">
+        <v>93</v>
+      </c>
+      <c r="C74">
+        <v>47.5</v>
+      </c>
+      <c r="D74">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A75">
+        <v>6</v>
+      </c>
+      <c r="B75" t="s">
+        <v>94</v>
+      </c>
+      <c r="C75">
+        <v>47.5</v>
+      </c>
+      <c r="D75">
+        <v>-6.5</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A76">
+        <v>6</v>
+      </c>
+      <c r="B76" t="s">
+        <v>95</v>
+      </c>
+      <c r="C76">
+        <v>46.5</v>
+      </c>
+      <c r="D76">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A77">
+        <v>6</v>
+      </c>
+      <c r="B77" t="s">
+        <v>96</v>
+      </c>
+      <c r="C77">
+        <v>51.5</v>
+      </c>
+      <c r="D77">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A78">
+        <v>6</v>
+      </c>
+      <c r="B78" t="s">
+        <v>97</v>
+      </c>
+      <c r="C78">
+        <v>50.5</v>
+      </c>
+      <c r="D78">
+        <v>5.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>